<commit_message>
updated excel with golden dataset result
</commit_message>
<xml_diff>
--- a/outputs/golden/golden_replay.xlsx
+++ b/outputs/golden/golden_replay.xlsx
@@ -1752,7 +1752,7 @@
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>Run: 2026-04-25 16:14</t>
+          <t>Run: 2026-04-26 13:08</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr"/>
@@ -1820,7 +1820,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-04-25 16:14</t>
+          <t>2026-04-26 13:08</t>
         </is>
       </c>
     </row>

</xml_diff>